<commit_message>
feat: route CRM imports by city
</commit_message>
<xml_diff>
--- a/docs/templates/algo-max-students-import-template.xlsx
+++ b/docs/templates/algo-max-students-import-template.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Инструкция" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Шаблон" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Инструкция" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Шаблон" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Инструкция'!$A$6:$D$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Шаблон'!$A$1:$J$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Инструкция'!$A$6:$D$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Шаблон'!$A$1:$L$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -460,7 +460,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D16"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -490,6 +490,13 @@
         </is>
       </c>
     </row>
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>По колонке «Город» строки автоматически распределяются между доступными вам городами. Все города должны быть заранее созданы в системе.</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
@@ -603,29 +610,29 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Группа</t>
+          <t>Дата рождения</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>Да</t>
+          <t>Нет</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Единое точное название группы</t>
+          <t>Дата рождения ученика в формате ДД.ММ.ГГГГ</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>1 3D общ вт 17:30 (год 25-26)</t>
+          <t>15.04.2015</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Курс</t>
+          <t>Город</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
@@ -635,19 +642,19 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Название учебного курса</t>
+          <t>Город ученика. Он должен быть заранее создан в Algo MAX</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Minecraft</t>
+          <t>Нижний Новгород</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Площадка</t>
+          <t>Группа</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -657,19 +664,19 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Адрес или название филиала</t>
+          <t>Единое точное название группы</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>Гагарина 64</t>
+          <t>1 3D общ вт 17:30 (год 25-26)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Преподаватель</t>
+          <t>Курс</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
@@ -679,65 +686,110 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>ФИО преподавателя как в его профиле</t>
+          <t>Название учебного курса</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Дворянинова Вероника</t>
+          <t>Minecraft</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>ID контакта</t>
+          <t>Площадка</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>Нет</t>
+          <t>Да</t>
         </is>
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>Contact ID родителя из amoCRM, не MAX ID</t>
+          <t>Адрес или название филиала</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>30420713</t>
+          <t>Гагарина 64</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Преподаватель</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Да</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>ФИО преподавателя как в его профиле</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Дворянинова Вероника</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>ID контакта</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>Нет</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Contact ID родителя из amoCRM, не MAX ID</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>30420713</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Имя контакта</t>
         </is>
       </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="B18" s="2" t="inlineStr">
         <is>
           <t>Нет</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>ФИО родителя</t>
         </is>
       </c>
-      <c r="D16" s="2" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Никина Елена Александровна</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:D16"/>
-  <mergeCells count="3">
+  <autoFilter ref="A6:D18"/>
+  <mergeCells count="4">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A4:D4"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A5:D5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -749,19 +801,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="34" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
     <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="34" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -787,37 +841,47 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
+          <t>Дата рождения</t>
+        </is>
+      </c>
+      <c r="F1" s="5" t="inlineStr">
+        <is>
+          <t>Город</t>
+        </is>
+      </c>
+      <c r="G1" s="5" t="inlineStr">
+        <is>
           <t>Группа</t>
         </is>
       </c>
-      <c r="F1" s="5" t="inlineStr">
+      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Курс</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
+      <c r="I1" s="5" t="inlineStr">
         <is>
           <t>Площадка</t>
         </is>
       </c>
-      <c r="H1" s="5" t="inlineStr">
+      <c r="J1" s="5" t="inlineStr">
         <is>
           <t>Преподаватель</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
+      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>ID контакта</t>
         </is>
       </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="L1" s="5" t="inlineStr">
         <is>
           <t>Имя контакта</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J1"/>
+  <autoFilter ref="A1:L1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>